<commit_message>
Reorganize tools and update sentence data
</commit_message>
<xml_diff>
--- a/vocab/review.xlsx
+++ b/vocab/review.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ICN00069\Downloads\scripts\vocab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{657C1FC1-6C8E-4F19-A4E7-21EDA6BF24F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{381E8190-115B-41F7-931F-06472CA4DF8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="A" sheetId="1" r:id="rId1"/>
@@ -24,6 +24,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">B!$C$1:$C$74</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'C'!$C$1:$C$129</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">D!$C$1:$C$74</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1034" uniqueCount="898">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1227" uniqueCount="927">
   <si>
     <t xml:space="preserve">aloof                 </t>
   </si>
@@ -2925,648 +2926,765 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>动物群</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>faze</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>使不安</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>feat</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>功绩</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>feather</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>羽毛</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>feces</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>feisty</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>充满精力的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fellow</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>小伙子</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fetus</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>胎儿</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>feud</t>
+  </si>
+  <si>
+    <t>世仇</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fictional</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>虚构的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fierce</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>（动作或情感）强烈的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fiery</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>燃烧的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>filial</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>孝顺的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>filth</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>污秽</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>finale</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>结局</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>峡湾</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fixture</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>固定装置</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>flame</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>火焰</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>flank</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>位于……的两侧</t>
+  </si>
+  <si>
+    <t>flatter</t>
+  </si>
+  <si>
+    <t>奉承</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>flea</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>跳蚤</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fleet</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>舰队</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fleshy</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>丰满的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>flex</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>弯曲</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fling</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>扔</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>flipper</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>鳍</t>
+  </si>
+  <si>
+    <t>flock</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>（鸟或羊等动物）群</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>floe</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>浮冰</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>floppy</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>松散下垂的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>flora</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>植物群</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>floss</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>牙线</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>flounder</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>挣扎</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fluff</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>绒毛</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>flute</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>长笛</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>focal</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>焦点的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>foe</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>敌人</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>foil</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>箔</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>forge</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>缔造</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>forsaken</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被抛弃的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fort</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>堡垒</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>forth</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>离去</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fortress</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>foul</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>难闻的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fragile</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>易碎的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>frail</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>人）脆弱的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fray</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>磨损</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>freakishly</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>反常地</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>frenzy</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>使发狂</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>friction</t>
+  </si>
+  <si>
+    <t>摩擦力</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fringe</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>穗，流苏；&lt;英&gt;刘海儿</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>frisky</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>活泼的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fro</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>来回的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>frolicking</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>嬉戏</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fromage</t>
+  </si>
+  <si>
+    <t>奶酪</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fume</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>发怒</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>funky</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>时髦的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fur</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>毛皮</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>furious</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>狂怒的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>furnish</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>为（房间或房屋）配备家具</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>furore</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>公愤</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fury</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>暴怒</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fuss</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>大惊小怪</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fuzz</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fuzzy</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>图片、声音等）不清楚的，模糊的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>aloof</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ambiance</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ammunition</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>amphibian</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>anal</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>anchovy</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>anemia</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>anemone</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>amnio</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Antarctica</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>antenna</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>古董</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>antique</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>aphrodisiac</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>appall</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>appoint</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>appraise</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>arbitray</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>arcade</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>archer</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>archipelago</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>arena</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>arid</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>armid</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>aroma</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>arnoist</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>动脉</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>arterial</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ascot</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ashore</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>assassin</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>assault</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>asteroid</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>atrium</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>asthma</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>attentive</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>专心的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>avocation</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>deny</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>deliquent</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>demean</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>dispicable</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>dicator</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>doogy</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>downbet</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>definace</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>fauna</t>
-  </si>
-  <si>
-    <t>动物群</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>faze</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>使不安</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>feat</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>功绩</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>feather</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>羽毛</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>feces</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>feisty</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>充满精力的</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>fellow</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>小伙子</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>fetus</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>胎儿</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>disceret</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>deinfect</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>dispostion</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>diggone</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>deridel</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>elegent</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>elite</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>elitism</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>engroged</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>entice</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>eternal</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>euphemism</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>exile</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>extoic</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>exploit</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>farbirication</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fanny</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>feud</t>
-  </si>
-  <si>
-    <t>世仇</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>fictional</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>虚构的</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>fierce</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>（动作或情感）强烈的</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>fiery</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>燃烧的</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>filial</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>孝顺的</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>filth</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>污秽</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>finale</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>结局</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>fiord</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>峡湾</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>fixture</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>固定装置</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>flame</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>火焰</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>flank</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>位于……的两侧</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fjord</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>flatter</t>
-  </si>
-  <si>
-    <t>奉承</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>flea</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>跳蚤</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>fleet</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>舰队</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>fleshy</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>丰满的</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>flex</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>弯曲</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>fling</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>扔</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>flipper</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>鳍</t>
-  </si>
-  <si>
-    <t>flock</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>（鸟或羊等动物）群</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>floe</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>浮冰</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>floppy</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>松散下垂的</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>flora</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>植物群</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>floss</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>牙线</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>flounder</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>挣扎</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>fluff</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>绒毛</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>flute</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>长笛</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>focal</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>焦点的</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>foe</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>敌人</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>foil</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>箔</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>forge</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>缔造</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>forsaken</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>被抛弃的</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>fort</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>堡垒</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>forth</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>离去</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>fortress</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>foul</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>难闻的</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>fragile</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>易碎的</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>frail</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>人）脆弱的</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>fray</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>磨损</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>freakishly</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>反常地</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>frenzy</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>使发狂</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>friction</t>
-  </si>
-  <si>
-    <t>摩擦力</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>fringe</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>穗，流苏；&lt;英&gt;刘海儿</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>frisky</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>活泼的</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>fro</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>来回的</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>frolicking</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>嬉戏</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>fromage</t>
-  </si>
-  <si>
-    <t>奶酪</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>fume</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>发怒</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>funky</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>时髦的</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>fur</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>毛皮</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>furious</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>狂怒的</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>furnish</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>为（房间或房屋）配备家具</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>furore</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>公愤</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>fury</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>暴怒</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>fuss</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>大惊小怪</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>fuzz</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>fuzzy</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>图片、声音等）不清楚的，模糊的</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>aloof</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>ambiance</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>ammunition</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>amphibian</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>anal</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>anchovy</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>anemia</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>anemone</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>amnio</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Antarctica</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>antenna</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>古董</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>antique</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>aphrodisiac</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>appall</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>appoint</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>appraise</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>arbitray</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>arcade</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>archer</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>archipelago</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>arena</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>arid</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>armid</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>aroma</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>arnoist</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>动脉</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>arterial</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>ascot</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>ashore</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>assassin</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>assault</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>asteroid</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>atrium</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>asthma</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>attentive</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>专心的</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>avocation</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -3574,7 +3692,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3601,12 +3719,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF101214"/>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -3628,7 +3740,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -3637,7 +3749,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3936,7 +4047,7 @@
   <dimension ref="A1:C36"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="21.5" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="10.4140625" customWidth="1"/>
     <col min="2" max="2" width="15.6640625" customWidth="1"/>
     <col min="3" max="3" width="15.08203125" customWidth="1"/>
   </cols>
@@ -3949,7 +4060,7 @@
         <v>181</v>
       </c>
       <c r="C1" t="s">
-        <v>860</v>
+        <v>858</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -3960,7 +4071,7 @@
         <v>182</v>
       </c>
       <c r="C2" t="s">
-        <v>861</v>
+        <v>859</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -3971,7 +4082,7 @@
         <v>183</v>
       </c>
       <c r="C3" t="s">
-        <v>862</v>
+        <v>860</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -3982,7 +4093,7 @@
         <v>184</v>
       </c>
       <c r="C4" t="s">
-        <v>868</v>
+        <v>866</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -3993,7 +4104,7 @@
         <v>185</v>
       </c>
       <c r="C5" t="s">
-        <v>863</v>
+        <v>861</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -4004,7 +4115,7 @@
         <v>186</v>
       </c>
       <c r="C6" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -4015,7 +4126,7 @@
         <v>187</v>
       </c>
       <c r="C7" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -4026,7 +4137,7 @@
         <v>188</v>
       </c>
       <c r="C8" t="s">
-        <v>866</v>
+        <v>864</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -4037,7 +4148,7 @@
         <v>189</v>
       </c>
       <c r="C9" t="s">
-        <v>867</v>
+        <v>865</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -4048,7 +4159,7 @@
         <v>190</v>
       </c>
       <c r="C10" t="s">
-        <v>869</v>
+        <v>867</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -4059,7 +4170,7 @@
         <v>192</v>
       </c>
       <c r="C11" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -4067,10 +4178,10 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
       <c r="C12" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -4081,7 +4192,7 @@
         <v>193</v>
       </c>
       <c r="C13" t="s">
-        <v>873</v>
+        <v>871</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -4092,7 +4203,7 @@
         <v>195</v>
       </c>
       <c r="C14" t="s">
-        <v>874</v>
+        <v>872</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -4103,7 +4214,7 @@
         <v>194</v>
       </c>
       <c r="C15" t="s">
-        <v>875</v>
+        <v>873</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -4114,7 +4225,7 @@
         <v>196</v>
       </c>
       <c r="C16" t="s">
-        <v>876</v>
+        <v>874</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -4125,7 +4236,7 @@
         <v>197</v>
       </c>
       <c r="C17" t="s">
-        <v>877</v>
+        <v>875</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -4136,7 +4247,7 @@
         <v>199</v>
       </c>
       <c r="C18" t="s">
-        <v>878</v>
+        <v>876</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -4147,7 +4258,7 @@
         <v>200</v>
       </c>
       <c r="C19" t="s">
-        <v>879</v>
+        <v>877</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -4158,7 +4269,7 @@
         <v>201</v>
       </c>
       <c r="C20" t="s">
-        <v>880</v>
+        <v>878</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -4169,7 +4280,7 @@
         <v>202</v>
       </c>
       <c r="C21" t="s">
-        <v>881</v>
+        <v>879</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -4180,7 +4291,7 @@
         <v>203</v>
       </c>
       <c r="C22" t="s">
-        <v>882</v>
+        <v>880</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -4191,7 +4302,7 @@
         <v>204</v>
       </c>
       <c r="C23" t="s">
-        <v>883</v>
+        <v>881</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -4202,7 +4313,7 @@
         <v>205</v>
       </c>
       <c r="C24" t="s">
-        <v>884</v>
+        <v>882</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -4213,7 +4324,7 @@
         <v>206</v>
       </c>
       <c r="C25" t="s">
-        <v>885</v>
+        <v>883</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -4221,10 +4332,10 @@
         <v>23</v>
       </c>
       <c r="B26" t="s">
-        <v>886</v>
+        <v>884</v>
       </c>
       <c r="C26" t="s">
-        <v>887</v>
+        <v>885</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -4235,7 +4346,7 @@
         <v>207</v>
       </c>
       <c r="C27" t="s">
-        <v>888</v>
+        <v>886</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -4246,7 +4357,7 @@
         <v>208</v>
       </c>
       <c r="C28" t="s">
-        <v>889</v>
+        <v>887</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -4257,7 +4368,7 @@
         <v>209</v>
       </c>
       <c r="C29" t="s">
-        <v>890</v>
+        <v>888</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -4268,7 +4379,7 @@
         <v>211</v>
       </c>
       <c r="C30" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -4279,7 +4390,7 @@
         <v>212</v>
       </c>
       <c r="C31" t="s">
-        <v>892</v>
+        <v>890</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -4290,7 +4401,7 @@
         <v>213</v>
       </c>
       <c r="C32" t="s">
-        <v>893</v>
+        <v>891</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -4301,7 +4412,7 @@
         <v>214</v>
       </c>
       <c r="C33" t="s">
-        <v>894</v>
+        <v>892</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -4309,10 +4420,10 @@
         <v>30</v>
       </c>
       <c r="B34" t="s">
-        <v>896</v>
+        <v>894</v>
       </c>
       <c r="C34" t="s">
-        <v>895</v>
+        <v>893</v>
       </c>
     </row>
     <row r="35" spans="1:3">
@@ -4323,7 +4434,7 @@
         <v>215</v>
       </c>
       <c r="C35" t="s">
-        <v>897</v>
+        <v>895</v>
       </c>
     </row>
     <row r="36" spans="1:3">
@@ -4367,9 +4478,7 @@
       <c r="B2" t="s">
         <v>40</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>175</v>
-      </c>
+      <c r="C2" s="3"/>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
@@ -6478,8 +6587,9 @@
   <dimension ref="A1:C74"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="14.9140625" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="16.5" customWidth="1"/>
     <col min="2" max="2" width="18.5" customWidth="1"/>
+    <col min="3" max="3" width="23.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -6500,6 +6610,9 @@
       <c r="B2" t="s">
         <v>478</v>
       </c>
+      <c r="C2" t="s">
+        <v>477</v>
+      </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
@@ -6508,6 +6621,9 @@
       <c r="B3" s="2" t="s">
         <v>480</v>
       </c>
+      <c r="C3" t="s">
+        <v>479</v>
+      </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
@@ -6516,6 +6632,9 @@
       <c r="B4" s="2" t="s">
         <v>482</v>
       </c>
+      <c r="C4" t="s">
+        <v>481</v>
+      </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
@@ -6524,6 +6643,9 @@
       <c r="B5" t="s">
         <v>484</v>
       </c>
+      <c r="C5" t="s">
+        <v>483</v>
+      </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
@@ -6532,6 +6654,9 @@
       <c r="B6" t="s">
         <v>486</v>
       </c>
+      <c r="C6" t="s">
+        <v>485</v>
+      </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
@@ -6540,6 +6665,9 @@
       <c r="B7" t="s">
         <v>488</v>
       </c>
+      <c r="C7" t="s">
+        <v>487</v>
+      </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
@@ -6548,6 +6676,9 @@
       <c r="B8" t="s">
         <v>490</v>
       </c>
+      <c r="C8" t="s">
+        <v>489</v>
+      </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
@@ -6556,6 +6687,9 @@
       <c r="B9" t="s">
         <v>492</v>
       </c>
+      <c r="C9" t="s">
+        <v>491</v>
+      </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
@@ -6564,6 +6698,9 @@
       <c r="B10" t="s">
         <v>494</v>
       </c>
+      <c r="C10" t="s">
+        <v>903</v>
+      </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
@@ -6572,6 +6709,9 @@
       <c r="B11" t="s">
         <v>496</v>
       </c>
+      <c r="C11" t="s">
+        <v>495</v>
+      </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
@@ -6580,6 +6720,9 @@
       <c r="B12" t="s">
         <v>498</v>
       </c>
+      <c r="C12" t="s">
+        <v>497</v>
+      </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
@@ -6588,6 +6731,9 @@
       <c r="B13" t="s">
         <v>500</v>
       </c>
+      <c r="C13" t="s">
+        <v>897</v>
+      </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
@@ -6596,6 +6742,9 @@
       <c r="B14" s="2" t="s">
         <v>502</v>
       </c>
+      <c r="C14" t="s">
+        <v>898</v>
+      </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
@@ -6604,6 +6753,9 @@
       <c r="B15" t="s">
         <v>504</v>
       </c>
+      <c r="C15" t="s">
+        <v>503</v>
+      </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
@@ -6612,868 +6764,1192 @@
       <c r="B16" t="s">
         <v>506</v>
       </c>
-    </row>
-    <row r="17" spans="1:2">
+      <c r="C16" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
       <c r="A17" t="s">
         <v>507</v>
       </c>
       <c r="B17" t="s">
         <v>508</v>
       </c>
-    </row>
-    <row r="18" spans="1:2">
+      <c r="C17" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
       <c r="A18" t="s">
         <v>509</v>
       </c>
       <c r="B18" t="s">
         <v>510</v>
       </c>
-    </row>
-    <row r="19" spans="1:2">
+      <c r="C18" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
       <c r="A19" t="s">
         <v>511</v>
       </c>
       <c r="B19" t="s">
         <v>512</v>
       </c>
-    </row>
-    <row r="20" spans="1:2">
+      <c r="C19" t="s">
+        <v>896</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
       <c r="A20" t="s">
         <v>513</v>
       </c>
       <c r="B20" t="s">
         <v>514</v>
       </c>
-    </row>
-    <row r="21" spans="1:2">
+      <c r="C20" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
       <c r="A21" t="s">
         <v>515</v>
       </c>
       <c r="B21" t="s">
         <v>516</v>
       </c>
-    </row>
-    <row r="22" spans="1:2">
+      <c r="C21" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
       <c r="A22" t="s">
         <v>517</v>
       </c>
       <c r="B22" t="s">
         <v>518</v>
       </c>
-    </row>
-    <row r="23" spans="1:2">
+      <c r="C22" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
       <c r="A23" t="s">
         <v>519</v>
       </c>
       <c r="B23" t="s">
         <v>520</v>
       </c>
-    </row>
-    <row r="24" spans="1:2">
+      <c r="C23" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
       <c r="A24" t="s">
         <v>521</v>
       </c>
       <c r="B24" t="s">
         <v>522</v>
       </c>
-    </row>
-    <row r="25" spans="1:2">
+      <c r="C24" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
       <c r="A25" t="s">
         <v>523</v>
       </c>
       <c r="B25" t="s">
         <v>524</v>
       </c>
-    </row>
-    <row r="26" spans="1:2">
+      <c r="C25" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
       <c r="A26" t="s">
         <v>525</v>
       </c>
       <c r="B26" t="s">
         <v>526</v>
       </c>
-    </row>
-    <row r="27" spans="1:2">
+      <c r="C26" t="s">
+        <v>899</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
       <c r="A27" t="s">
         <v>527</v>
       </c>
       <c r="B27" t="s">
         <v>528</v>
       </c>
-    </row>
-    <row r="28" spans="1:2">
+      <c r="C27" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
       <c r="A28" t="s">
         <v>529</v>
       </c>
       <c r="B28" t="s">
         <v>530</v>
       </c>
-    </row>
-    <row r="29" spans="1:2">
+      <c r="C28" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
       <c r="A29" t="s">
         <v>531</v>
       </c>
       <c r="B29" t="s">
         <v>532</v>
       </c>
-    </row>
-    <row r="30" spans="1:2">
+      <c r="C29" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
       <c r="A30" t="s">
         <v>533</v>
       </c>
       <c r="B30" t="s">
         <v>534</v>
       </c>
-    </row>
-    <row r="31" spans="1:2">
+      <c r="C30" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
       <c r="A31" t="s">
         <v>535</v>
       </c>
       <c r="B31" t="s">
         <v>536</v>
       </c>
-    </row>
-    <row r="32" spans="1:2">
+      <c r="C31" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
       <c r="A32" t="s">
         <v>537</v>
       </c>
       <c r="B32" t="s">
         <v>538</v>
       </c>
-    </row>
-    <row r="33" spans="1:2">
+      <c r="C32" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
       <c r="A33" t="s">
         <v>539</v>
       </c>
       <c r="B33" t="s">
         <v>540</v>
       </c>
-    </row>
-    <row r="34" spans="1:2">
+      <c r="C33" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
       <c r="A34" t="s">
         <v>541</v>
       </c>
       <c r="B34" t="s">
         <v>542</v>
       </c>
-    </row>
-    <row r="35" spans="1:2">
+      <c r="C34" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
       <c r="A35" t="s">
         <v>543</v>
       </c>
       <c r="B35" t="s">
         <v>544</v>
       </c>
-    </row>
-    <row r="36" spans="1:2">
+      <c r="C35" t="s">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
       <c r="A36" t="s">
         <v>545</v>
       </c>
       <c r="B36" t="s">
         <v>546</v>
       </c>
-    </row>
-    <row r="37" spans="1:2">
+      <c r="C36" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
       <c r="A37" t="s">
         <v>547</v>
       </c>
       <c r="B37" t="s">
         <v>548</v>
       </c>
-    </row>
-    <row r="38" spans="1:2">
+      <c r="C37" s="3" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
       <c r="A38" t="s">
         <v>549</v>
       </c>
       <c r="B38" t="s">
         <v>550</v>
       </c>
-    </row>
-    <row r="39" spans="1:2">
+      <c r="C38" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
       <c r="A39" t="s">
         <v>551</v>
       </c>
       <c r="B39" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="40" spans="1:2">
+      <c r="C39" t="s">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
       <c r="A40" t="s">
         <v>553</v>
       </c>
       <c r="B40" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="41" spans="1:2">
+      <c r="C40" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
       <c r="A41" t="s">
         <v>554</v>
       </c>
       <c r="B41" t="s">
         <v>555</v>
       </c>
-    </row>
-    <row r="42" spans="1:2">
+      <c r="C41" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
       <c r="A42" t="s">
         <v>556</v>
       </c>
       <c r="B42" t="s">
         <v>557</v>
       </c>
-    </row>
-    <row r="43" spans="1:2">
+      <c r="C42" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
       <c r="A43" t="s">
         <v>558</v>
       </c>
       <c r="B43" t="s">
         <v>559</v>
       </c>
-    </row>
-    <row r="44" spans="1:2">
+      <c r="C43" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
       <c r="A44" t="s">
         <v>560</v>
       </c>
       <c r="B44" t="s">
         <v>561</v>
       </c>
-    </row>
-    <row r="45" spans="1:2">
+      <c r="C44" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
       <c r="A45" t="s">
         <v>562</v>
       </c>
       <c r="B45" t="s">
         <v>563</v>
       </c>
-    </row>
-    <row r="46" spans="1:2">
+      <c r="C45" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3">
       <c r="A46" t="s">
         <v>564</v>
       </c>
       <c r="B46" t="s">
         <v>565</v>
       </c>
-    </row>
-    <row r="47" spans="1:2">
+      <c r="C46" t="s">
+        <v>905</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3">
       <c r="A47" t="s">
         <v>566</v>
       </c>
       <c r="B47" t="s">
         <v>567</v>
       </c>
-    </row>
-    <row r="48" spans="1:2">
+      <c r="C47" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3">
       <c r="A48" t="s">
         <v>568</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>569</v>
       </c>
-    </row>
-    <row r="49" spans="1:2">
+      <c r="C48" t="s">
+        <v>906</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3">
       <c r="A49" t="s">
         <v>570</v>
       </c>
       <c r="B49" t="s">
         <v>571</v>
       </c>
-    </row>
-    <row r="50" spans="1:2">
+      <c r="C49" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3">
       <c r="A50" t="s">
         <v>572</v>
       </c>
       <c r="B50" t="s">
         <v>573</v>
       </c>
-    </row>
-    <row r="51" spans="1:2">
+      <c r="C50" t="s">
+        <v>907</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3">
       <c r="A51" t="s">
         <v>574</v>
       </c>
       <c r="B51" t="s">
         <v>575</v>
       </c>
-    </row>
-    <row r="52" spans="1:2">
+      <c r="C51" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3">
       <c r="A52" t="s">
         <v>576</v>
       </c>
       <c r="B52" t="s">
         <v>577</v>
       </c>
-    </row>
-    <row r="53" spans="1:2">
+      <c r="C52" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3">
       <c r="A53" t="s">
         <v>578</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>579</v>
       </c>
-    </row>
-    <row r="54" spans="1:2">
+      <c r="C53" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3">
       <c r="A54" t="s">
         <v>580</v>
       </c>
       <c r="B54" t="s">
         <v>581</v>
       </c>
-    </row>
-    <row r="55" spans="1:2">
+      <c r="C54" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3">
       <c r="A55" t="s">
         <v>582</v>
       </c>
       <c r="B55" t="s">
         <v>583</v>
       </c>
-    </row>
-    <row r="56" spans="1:2">
+      <c r="C55" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3">
       <c r="A56" t="s">
         <v>584</v>
       </c>
       <c r="B56" t="s">
         <v>585</v>
       </c>
-    </row>
-    <row r="57" spans="1:2">
+      <c r="C56" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3">
       <c r="A57" t="s">
         <v>586</v>
       </c>
       <c r="B57" t="s">
         <v>587</v>
       </c>
-    </row>
-    <row r="58" spans="1:2">
+      <c r="C57" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3">
       <c r="A58" t="s">
         <v>588</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>589</v>
       </c>
-    </row>
-    <row r="59" spans="1:2">
+      <c r="C58" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3">
       <c r="A59" t="s">
         <v>590</v>
       </c>
       <c r="B59" t="s">
         <v>462</v>
       </c>
-    </row>
-    <row r="60" spans="1:2">
+      <c r="C59" t="s">
+        <v>901</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3">
       <c r="A60" t="s">
         <v>591</v>
       </c>
       <c r="B60" t="s">
         <v>592</v>
       </c>
-    </row>
-    <row r="61" spans="1:2">
+      <c r="C60" t="s">
+        <v>908</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3">
       <c r="A61" t="s">
         <v>593</v>
       </c>
       <c r="B61" t="s">
         <v>594</v>
       </c>
-    </row>
-    <row r="62" spans="1:2">
+      <c r="C61" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3">
       <c r="A62" t="s">
         <v>595</v>
       </c>
       <c r="B62" t="s">
         <v>596</v>
       </c>
-    </row>
-    <row r="63" spans="1:2">
+      <c r="C62" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3">
       <c r="A63" t="s">
         <v>597</v>
       </c>
       <c r="B63" t="s">
         <v>598</v>
       </c>
-    </row>
-    <row r="64" spans="1:2">
+      <c r="C63" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3">
       <c r="A64" t="s">
         <v>599</v>
       </c>
       <c r="B64" t="s">
         <v>600</v>
       </c>
-    </row>
-    <row r="65" spans="1:2">
+      <c r="C64" t="s">
+        <v>902</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3">
       <c r="A65" t="s">
         <v>601</v>
       </c>
       <c r="B65" t="s">
         <v>602</v>
       </c>
-    </row>
-    <row r="66" spans="1:2">
+      <c r="C65" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3">
       <c r="A66" t="s">
         <v>603</v>
       </c>
       <c r="B66" t="s">
         <v>604</v>
       </c>
-    </row>
-    <row r="67" spans="1:2">
+      <c r="C66" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3">
       <c r="A67" t="s">
         <v>605</v>
       </c>
       <c r="B67" t="s">
         <v>606</v>
       </c>
-    </row>
-    <row r="68" spans="1:2">
+      <c r="C67" t="s">
+        <v>909</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3">
       <c r="A68" t="s">
         <v>607</v>
       </c>
       <c r="B68" t="s">
         <v>608</v>
       </c>
-    </row>
-    <row r="69" spans="1:2">
+      <c r="C68" t="s">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3">
       <c r="A69" t="s">
         <v>609</v>
       </c>
       <c r="B69" t="s">
         <v>610</v>
       </c>
-    </row>
-    <row r="70" spans="1:2">
+      <c r="C69" t="s">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3">
       <c r="A70" t="s">
         <v>611</v>
       </c>
       <c r="B70" t="s">
         <v>612</v>
       </c>
-    </row>
-    <row r="71" spans="1:2">
+      <c r="C70" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3">
       <c r="A71" t="s">
         <v>613</v>
       </c>
       <c r="B71" t="s">
         <v>614</v>
       </c>
-    </row>
-    <row r="72" spans="1:2">
+      <c r="C71" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3">
       <c r="A72" t="s">
         <v>615</v>
       </c>
       <c r="B72" t="s">
         <v>616</v>
       </c>
-    </row>
-    <row r="73" spans="1:2">
+      <c r="C72" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3">
       <c r="A73" t="s">
         <v>617</v>
       </c>
       <c r="B73" t="s">
         <v>618</v>
       </c>
-    </row>
-    <row r="74" spans="1:2">
+      <c r="C73" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3">
       <c r="A74" t="s">
         <v>619</v>
       </c>
       <c r="B74" t="s">
         <v>620</v>
       </c>
+      <c r="C74" t="s">
+        <v>619</v>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="C1:C74" xr:uid="{F1CCD6F2-B6CD-4EE2-92A8-4F202D19A46B}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0766560D-3EEC-421C-A0AF-B5DEB320A4E4}">
-  <dimension ref="A1:B48"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="20.5" customWidth="1"/>
     <col min="2" max="2" width="13.83203125" customWidth="1"/>
+    <col min="3" max="3" width="13.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>621</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>622</v>
       </c>
-    </row>
-    <row r="2" spans="1:2">
+      <c r="C1" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>623</v>
       </c>
       <c r="B2" t="s">
         <v>624</v>
       </c>
-    </row>
-    <row r="3" spans="1:2">
+      <c r="C2" t="s">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>625</v>
       </c>
       <c r="B3" t="s">
         <v>626</v>
       </c>
-    </row>
-    <row r="4" spans="1:2">
+      <c r="C3" t="s">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>627</v>
       </c>
       <c r="B4" t="s">
         <v>628</v>
       </c>
-    </row>
-    <row r="5" spans="1:2">
+      <c r="C4" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>629</v>
       </c>
       <c r="B5" t="s">
         <v>630</v>
       </c>
-    </row>
-    <row r="6" spans="1:2">
+      <c r="C5" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>631</v>
       </c>
       <c r="B6" t="s">
         <v>632</v>
       </c>
-    </row>
-    <row r="7" spans="1:2">
+      <c r="C6" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>633</v>
       </c>
       <c r="B7" t="s">
         <v>634</v>
       </c>
-    </row>
-    <row r="8" spans="1:2">
+      <c r="C7" t="s">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>635</v>
       </c>
       <c r="B8" t="s">
         <v>636</v>
       </c>
-    </row>
-    <row r="9" spans="1:2">
+      <c r="C8" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>637</v>
       </c>
       <c r="B9" t="s">
         <v>638</v>
       </c>
-    </row>
-    <row r="10" spans="1:2">
+      <c r="C9" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
       <c r="A10" t="s">
         <v>639</v>
       </c>
       <c r="B10" t="s">
         <v>640</v>
       </c>
-    </row>
-    <row r="11" spans="1:2">
+      <c r="C10" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
       <c r="A11" t="s">
         <v>641</v>
       </c>
       <c r="B11" t="s">
         <v>642</v>
       </c>
-    </row>
-    <row r="12" spans="1:2">
+      <c r="C11" t="s">
+        <v>911</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
       <c r="A12" t="s">
         <v>643</v>
       </c>
       <c r="B12" t="s">
         <v>644</v>
       </c>
-    </row>
-    <row r="13" spans="1:2">
+      <c r="C12" t="s">
+        <v>912</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
       <c r="A13" t="s">
         <v>645</v>
       </c>
       <c r="B13" t="s">
         <v>646</v>
       </c>
-    </row>
-    <row r="14" spans="1:2">
+      <c r="C13" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>647</v>
       </c>
       <c r="B14" t="s">
         <v>648</v>
       </c>
-    </row>
-    <row r="15" spans="1:2">
+      <c r="C14" t="s">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
       <c r="A15" t="s">
         <v>649</v>
       </c>
       <c r="B15" t="s">
         <v>650</v>
       </c>
-    </row>
-    <row r="16" spans="1:2">
+      <c r="C15" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
       <c r="A16" t="s">
         <v>651</v>
       </c>
       <c r="B16" t="s">
         <v>652</v>
       </c>
-    </row>
-    <row r="17" spans="1:2">
+      <c r="C16" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
       <c r="A17" t="s">
         <v>653</v>
       </c>
       <c r="B17" t="s">
         <v>654</v>
       </c>
-    </row>
-    <row r="18" spans="1:2">
+      <c r="C17" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
       <c r="A18" t="s">
         <v>655</v>
       </c>
       <c r="B18" t="s">
         <v>656</v>
       </c>
-    </row>
-    <row r="19" spans="1:2">
+      <c r="C18" t="s">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
       <c r="A19" t="s">
         <v>657</v>
       </c>
       <c r="B19" t="s">
         <v>658</v>
       </c>
-    </row>
-    <row r="20" spans="1:2">
+      <c r="C19" t="s">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
       <c r="A20" t="s">
         <v>659</v>
       </c>
       <c r="B20" t="s">
         <v>660</v>
       </c>
-    </row>
-    <row r="21" spans="1:2">
+      <c r="C20" t="s">
+        <v>913</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
       <c r="A21" t="s">
         <v>661</v>
       </c>
       <c r="B21" t="s">
         <v>662</v>
       </c>
-    </row>
-    <row r="22" spans="1:2">
+      <c r="C21" t="s">
+        <v>661</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
       <c r="A22" t="s">
         <v>663</v>
       </c>
       <c r="B22" t="s">
         <v>664</v>
       </c>
-    </row>
-    <row r="23" spans="1:2">
+      <c r="C22" t="s">
+        <v>914</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
       <c r="A23" t="s">
         <v>665</v>
       </c>
       <c r="B23" t="s">
         <v>666</v>
       </c>
-    </row>
-    <row r="24" spans="1:2">
+      <c r="C23" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
       <c r="A24" t="s">
         <v>667</v>
       </c>
       <c r="B24" t="s">
         <v>668</v>
       </c>
-    </row>
-    <row r="25" spans="1:2">
+      <c r="C24" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
       <c r="A25" t="s">
         <v>669</v>
       </c>
       <c r="B25" t="s">
         <v>670</v>
       </c>
-    </row>
-    <row r="26" spans="1:2">
+      <c r="C25" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
       <c r="A26" t="s">
         <v>671</v>
       </c>
       <c r="B26" t="s">
         <v>672</v>
       </c>
-    </row>
-    <row r="27" spans="1:2">
+      <c r="C26" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
       <c r="A27" t="s">
         <v>673</v>
       </c>
       <c r="B27" t="s">
         <v>674</v>
       </c>
-    </row>
-    <row r="28" spans="1:2">
+      <c r="C27" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
       <c r="A28" t="s">
         <v>675</v>
       </c>
       <c r="B28" t="s">
         <v>676</v>
       </c>
-    </row>
-    <row r="29" spans="1:2">
+      <c r="C28" t="s">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
       <c r="A29" t="s">
         <v>677</v>
       </c>
       <c r="B29" t="s">
         <v>678</v>
       </c>
-    </row>
-    <row r="30" spans="1:2">
+      <c r="C29" t="s">
+        <v>677</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
       <c r="A30" t="s">
         <v>679</v>
       </c>
       <c r="B30" t="s">
         <v>680</v>
       </c>
-    </row>
-    <row r="31" spans="1:2">
+      <c r="C30" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
       <c r="A31" t="s">
         <v>681</v>
       </c>
       <c r="B31" t="s">
         <v>682</v>
       </c>
-    </row>
-    <row r="32" spans="1:2">
+      <c r="C31" t="s">
+        <v>681</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
       <c r="A32" t="s">
         <v>683</v>
       </c>
       <c r="B32" t="s">
         <v>684</v>
       </c>
-    </row>
-    <row r="33" spans="1:2">
+      <c r="C32" t="s">
+        <v>915</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
       <c r="A33" t="s">
         <v>685</v>
       </c>
       <c r="B33" t="s">
         <v>686</v>
       </c>
-    </row>
-    <row r="34" spans="1:2">
+      <c r="C33" t="s">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
       <c r="A34" t="s">
         <v>687</v>
       </c>
       <c r="B34" t="s">
         <v>688</v>
       </c>
-    </row>
-    <row r="35" spans="1:2">
+      <c r="C34" t="s">
+        <v>916</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
       <c r="A35" t="s">
         <v>689</v>
       </c>
       <c r="B35" t="s">
         <v>690</v>
       </c>
-    </row>
-    <row r="36" spans="1:2">
+      <c r="C35" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
       <c r="A36" t="s">
         <v>691</v>
       </c>
       <c r="B36" t="s">
         <v>692</v>
       </c>
-    </row>
-    <row r="37" spans="1:2">
+      <c r="C36" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
       <c r="A37" t="s">
         <v>693</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>694</v>
       </c>
-    </row>
-    <row r="38" spans="1:2">
+      <c r="C37" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
       <c r="A38" t="s">
         <v>695</v>
       </c>
       <c r="B38" t="s">
         <v>696</v>
       </c>
-    </row>
-    <row r="39" spans="1:2">
+      <c r="C38" t="s">
+        <v>917</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
       <c r="A39" t="s">
         <v>697</v>
       </c>
       <c r="B39" t="s">
         <v>698</v>
       </c>
-    </row>
-    <row r="40" spans="1:2">
+      <c r="C39" t="s">
+        <v>918</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
       <c r="A40" t="s">
         <v>699</v>
       </c>
       <c r="B40" t="s">
         <v>700</v>
       </c>
-    </row>
-    <row r="41" spans="1:2">
+      <c r="C40" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
       <c r="A41" t="s">
         <v>701</v>
       </c>
       <c r="B41" t="s">
         <v>702</v>
       </c>
-    </row>
-    <row r="42" spans="1:2">
+      <c r="C41" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
       <c r="A42" t="s">
         <v>703</v>
       </c>
       <c r="B42" t="s">
         <v>704</v>
       </c>
-    </row>
-    <row r="43" spans="1:2">
+      <c r="C42" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
       <c r="A43" t="s">
         <v>705</v>
       </c>
       <c r="B43" t="s">
         <v>706</v>
       </c>
-    </row>
-    <row r="44" spans="1:2">
+      <c r="C43" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
       <c r="A44" t="s">
         <v>707</v>
       </c>
       <c r="B44" t="s">
         <v>708</v>
       </c>
-    </row>
-    <row r="45" spans="1:2">
+      <c r="C44" t="s">
+        <v>919</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
       <c r="A45" t="s">
         <v>709</v>
       </c>
       <c r="B45" t="s">
         <v>710</v>
       </c>
-    </row>
-    <row r="46" spans="1:2">
+      <c r="C45" t="s">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3">
       <c r="A46" t="s">
         <v>711</v>
       </c>
       <c r="B46" t="s">
         <v>712</v>
       </c>
-    </row>
-    <row r="47" spans="1:2">
+      <c r="C46" t="s">
+        <v>711</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3">
       <c r="A47" t="s">
         <v>713</v>
       </c>
       <c r="B47" t="s">
         <v>714</v>
       </c>
-    </row>
-    <row r="48" spans="1:2">
+      <c r="C47" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3">
       <c r="A48" t="s">
         <v>715</v>
       </c>
       <c r="B48" t="s">
         <v>716</v>
+      </c>
+      <c r="C48" t="s">
+        <v>715</v>
       </c>
     </row>
   </sheetData>
@@ -7484,595 +7960,815 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A440402-F3E7-4453-8C1F-54B73D95329A}">
-  <dimension ref="A1:B73"/>
+  <dimension ref="A1:C73"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="19.33203125" customWidth="1"/>
-    <col min="2" max="2" width="24.9140625" customWidth="1"/>
+    <col min="2" max="2" width="33.08203125" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>717</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>718</v>
       </c>
-    </row>
-    <row r="2" spans="1:2">
+      <c r="C1" t="s">
+        <v>920</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>719</v>
       </c>
       <c r="B2" t="s">
         <v>720</v>
       </c>
-    </row>
-    <row r="3" spans="1:2">
+      <c r="C2" t="s">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>721</v>
       </c>
       <c r="B3" t="s">
         <v>722</v>
       </c>
-    </row>
-    <row r="4" spans="1:2">
+      <c r="C3" t="s">
+        <v>721</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>723</v>
       </c>
       <c r="B4" t="s">
         <v>724</v>
       </c>
-    </row>
-    <row r="5" spans="1:2">
+      <c r="C4" t="s">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>725</v>
       </c>
       <c r="B5" t="s">
         <v>726</v>
       </c>
-    </row>
-    <row r="6" spans="1:2">
+      <c r="C5" t="s">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>727</v>
       </c>
       <c r="B6" t="s">
         <v>728</v>
       </c>
-    </row>
-    <row r="7" spans="1:2">
+      <c r="C6" t="s">
+        <v>921</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>729</v>
       </c>
       <c r="B7" t="s">
         <v>730</v>
       </c>
-    </row>
-    <row r="8" spans="1:2">
+      <c r="C7" t="s">
+        <v>729</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>731</v>
       </c>
       <c r="B8" t="s">
         <v>732</v>
       </c>
-    </row>
-    <row r="9" spans="1:2">
+      <c r="C8" t="s">
+        <v>731</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>733</v>
       </c>
       <c r="B9" t="s">
         <v>734</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" ht="17.5">
-      <c r="A10" s="4" t="s">
+      <c r="C9" t="s">
+        <v>733</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>904</v>
+      </c>
+      <c r="B10" t="s">
         <v>735</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
         <v>736</v>
       </c>
-    </row>
-    <row r="11" spans="1:2">
-      <c r="A11" t="s">
+      <c r="B11" t="s">
         <v>737</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" t="s">
         <v>738</v>
       </c>
-    </row>
-    <row r="12" spans="1:2">
-      <c r="A12" t="s">
+      <c r="B12" t="s">
         <v>739</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" t="s">
         <v>740</v>
       </c>
-    </row>
-    <row r="13" spans="1:2">
-      <c r="A13" t="s">
+      <c r="B13" t="s">
         <v>741</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" t="s">
         <v>742</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2">
-      <c r="A14" t="s">
-        <v>743</v>
       </c>
       <c r="B14" t="s">
         <v>594</v>
       </c>
-    </row>
-    <row r="15" spans="1:2">
+      <c r="C14" t="s">
+        <v>742</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
       <c r="A15" t="s">
+        <v>743</v>
+      </c>
+      <c r="B15" t="s">
         <v>744</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" t="s">
         <v>745</v>
       </c>
-    </row>
-    <row r="16" spans="1:2">
-      <c r="A16" t="s">
+      <c r="B16" t="s">
         <v>746</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" t="s">
         <v>747</v>
       </c>
-    </row>
-    <row r="17" spans="1:2">
-      <c r="A17" t="s">
+      <c r="B17" t="s">
         <v>748</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
+        <v>747</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" t="s">
         <v>749</v>
       </c>
-    </row>
-    <row r="18" spans="1:2">
-      <c r="A18" t="s">
+      <c r="B18" t="s">
         <v>750</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
+        <v>922</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" t="s">
         <v>751</v>
       </c>
-    </row>
-    <row r="19" spans="1:2">
-      <c r="A19" t="s">
+      <c r="B19" t="s">
         <v>752</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" t="s">
         <v>753</v>
       </c>
-    </row>
-    <row r="20" spans="1:2">
-      <c r="A20" t="s">
+      <c r="B20" t="s">
         <v>754</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" t="s">
         <v>755</v>
       </c>
-    </row>
-    <row r="21" spans="1:2">
-      <c r="A21" t="s">
+      <c r="B21" t="s">
         <v>756</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" t="s">
         <v>757</v>
       </c>
-    </row>
-    <row r="22" spans="1:2">
-      <c r="A22" t="s">
+      <c r="B22" t="s">
         <v>758</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" t="s">
         <v>759</v>
       </c>
-    </row>
-    <row r="23" spans="1:2">
-      <c r="A23" t="s">
+      <c r="B23" t="s">
         <v>760</v>
       </c>
-      <c r="B23" t="s">
+      <c r="C23" t="s">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" t="s">
         <v>761</v>
       </c>
-    </row>
-    <row r="24" spans="1:2">
-      <c r="A24" t="s">
+      <c r="B24" t="s">
         <v>762</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" t="s">
+        <v>923</v>
+      </c>
+      <c r="B25" t="s">
         <v>763</v>
       </c>
-    </row>
-    <row r="25" spans="1:2">
-      <c r="A25" t="s">
+      <c r="C25" t="s">
+        <v>923</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" t="s">
         <v>764</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B26" t="s">
         <v>765</v>
       </c>
-    </row>
-    <row r="26" spans="1:2">
-      <c r="A26" t="s">
+      <c r="C26" t="s">
+        <v>764</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27" t="s">
         <v>766</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B27" t="s">
         <v>767</v>
       </c>
-    </row>
-    <row r="27" spans="1:2">
-      <c r="A27" t="s">
+      <c r="C27" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="A28" t="s">
         <v>768</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B28" t="s">
         <v>769</v>
       </c>
-    </row>
-    <row r="28" spans="1:2">
-      <c r="A28" t="s">
+      <c r="C28" t="s">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29" t="s">
         <v>770</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B29" t="s">
         <v>771</v>
       </c>
-    </row>
-    <row r="29" spans="1:2">
-      <c r="A29" t="s">
+      <c r="C29" t="s">
+        <v>924</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" t="s">
         <v>772</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B30" t="s">
         <v>773</v>
       </c>
-    </row>
-    <row r="30" spans="1:2">
-      <c r="A30" t="s">
+      <c r="C30" t="s">
+        <v>772</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" t="s">
         <v>774</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B31" t="s">
         <v>775</v>
       </c>
-    </row>
-    <row r="31" spans="1:2">
-      <c r="A31" t="s">
+      <c r="C31" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" t="s">
         <v>776</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B32" t="s">
         <v>777</v>
       </c>
-    </row>
-    <row r="32" spans="1:2">
-      <c r="A32" t="s">
+      <c r="C32" t="s">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" t="s">
         <v>778</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B33" t="s">
         <v>779</v>
       </c>
-    </row>
-    <row r="33" spans="1:2">
-      <c r="A33" t="s">
+      <c r="C33" t="s">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" t="s">
         <v>780</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B34" t="s">
         <v>781</v>
       </c>
-    </row>
-    <row r="34" spans="1:2">
-      <c r="A34" t="s">
+      <c r="C34" t="s">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" t="s">
         <v>782</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B35" t="s">
         <v>783</v>
       </c>
-    </row>
-    <row r="35" spans="1:2">
-      <c r="A35" t="s">
+      <c r="C35" t="s">
+        <v>782</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" t="s">
         <v>784</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B36" t="s">
         <v>785</v>
       </c>
-    </row>
-    <row r="36" spans="1:2">
-      <c r="A36" t="s">
+      <c r="C36" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37" t="s">
         <v>786</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B37" t="s">
         <v>787</v>
       </c>
-    </row>
-    <row r="37" spans="1:2">
-      <c r="A37" t="s">
+      <c r="C37" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" t="s">
         <v>788</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B38" t="s">
         <v>789</v>
       </c>
-    </row>
-    <row r="38" spans="1:2">
-      <c r="A38" t="s">
+      <c r="C38" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" t="s">
         <v>790</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B39" t="s">
         <v>791</v>
       </c>
-    </row>
-    <row r="39" spans="1:2">
-      <c r="A39" t="s">
+      <c r="C39" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" t="s">
         <v>792</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B40" t="s">
         <v>793</v>
       </c>
-    </row>
-    <row r="40" spans="1:2">
-      <c r="A40" t="s">
+      <c r="C40" t="s">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41" t="s">
         <v>794</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B41" t="s">
         <v>795</v>
       </c>
-    </row>
-    <row r="41" spans="1:2">
-      <c r="A41" t="s">
+      <c r="C41" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
+      <c r="A42" t="s">
         <v>796</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B42" t="s">
         <v>797</v>
       </c>
-    </row>
-    <row r="42" spans="1:2">
-      <c r="A42" t="s">
+      <c r="C42" t="s">
+        <v>796</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="A43" t="s">
         <v>798</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B43" t="s">
         <v>799</v>
       </c>
-    </row>
-    <row r="43" spans="1:2">
-      <c r="A43" t="s">
+      <c r="C43" t="s">
+        <v>798</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
+      <c r="A44" t="s">
         <v>800</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B44" t="s">
         <v>801</v>
       </c>
-    </row>
-    <row r="44" spans="1:2">
-      <c r="A44" t="s">
+      <c r="C44" t="s">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
+      <c r="A45" t="s">
         <v>802</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B45" t="s">
         <v>803</v>
       </c>
-    </row>
-    <row r="45" spans="1:2">
-      <c r="A45" t="s">
+      <c r="C45" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3">
+      <c r="A46" t="s">
         <v>804</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B46" t="s">
         <v>805</v>
       </c>
-    </row>
-    <row r="46" spans="1:2">
-      <c r="A46" t="s">
+      <c r="C46" t="s">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3">
+      <c r="A47" t="s">
         <v>806</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B47" t="s">
         <v>807</v>
       </c>
-    </row>
-    <row r="47" spans="1:2">
-      <c r="A47" t="s">
+      <c r="C47" t="s">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3">
+      <c r="A48" t="s">
         <v>808</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B48" t="s">
         <v>809</v>
       </c>
-    </row>
-    <row r="48" spans="1:2">
-      <c r="A48" t="s">
+      <c r="C48" t="s">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3">
+      <c r="A49" t="s">
         <v>810</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B49" t="s">
         <v>811</v>
       </c>
-    </row>
-    <row r="49" spans="1:2">
-      <c r="A49" t="s">
+      <c r="C49" t="s">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3">
+      <c r="A50" t="s">
         <v>812</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B50" t="s">
         <v>813</v>
       </c>
-    </row>
-    <row r="50" spans="1:2">
-      <c r="A50" t="s">
+      <c r="C50" t="s">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3">
+      <c r="A51" t="s">
         <v>814</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B51" t="s">
+        <v>811</v>
+      </c>
+      <c r="C51" t="s">
+        <v>814</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3">
+      <c r="A52" t="s">
         <v>815</v>
       </c>
-    </row>
-    <row r="51" spans="1:2">
-      <c r="A51" t="s">
+      <c r="B52" t="s">
         <v>816</v>
       </c>
-      <c r="B51" t="s">
-        <v>813</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2">
-      <c r="A52" t="s">
+      <c r="C52" t="s">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3">
+      <c r="A53" t="s">
         <v>817</v>
       </c>
-      <c r="B52" t="s">
+      <c r="B53" t="s">
         <v>818</v>
       </c>
-    </row>
-    <row r="53" spans="1:2">
-      <c r="A53" t="s">
+      <c r="C53" t="s">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3">
+      <c r="A54" t="s">
         <v>819</v>
       </c>
-      <c r="B53" t="s">
+      <c r="B54" t="s">
         <v>820</v>
       </c>
-    </row>
-    <row r="54" spans="1:2">
-      <c r="A54" t="s">
+      <c r="C54" t="s">
+        <v>819</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3">
+      <c r="A55" t="s">
         <v>821</v>
       </c>
-      <c r="B54" t="s">
+      <c r="B55" t="s">
         <v>822</v>
       </c>
-    </row>
-    <row r="55" spans="1:2">
-      <c r="A55" t="s">
+      <c r="C55" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3">
+      <c r="A56" t="s">
         <v>823</v>
       </c>
-      <c r="B55" t="s">
+      <c r="B56" t="s">
         <v>824</v>
       </c>
-    </row>
-    <row r="56" spans="1:2">
-      <c r="A56" t="s">
+      <c r="C56" t="s">
+        <v>823</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3">
+      <c r="A57" t="s">
         <v>825</v>
       </c>
-      <c r="B56" t="s">
+      <c r="B57" t="s">
         <v>826</v>
       </c>
-    </row>
-    <row r="57" spans="1:2">
-      <c r="A57" t="s">
+      <c r="C57" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3">
+      <c r="A58" t="s">
         <v>827</v>
       </c>
-      <c r="B57" t="s">
+      <c r="B58" t="s">
         <v>828</v>
       </c>
-    </row>
-    <row r="58" spans="1:2">
-      <c r="A58" t="s">
+      <c r="C58" t="s">
+        <v>925</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3">
+      <c r="A59" t="s">
         <v>829</v>
       </c>
-      <c r="B58" t="s">
+      <c r="B59" s="2" t="s">
         <v>830</v>
       </c>
-    </row>
-    <row r="59" spans="1:2">
-      <c r="A59" t="s">
+      <c r="C59" t="s">
+        <v>829</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3">
+      <c r="A60" t="s">
         <v>831</v>
       </c>
-      <c r="B59" s="2" t="s">
+      <c r="B60" t="s">
         <v>832</v>
       </c>
-    </row>
-    <row r="60" spans="1:2">
-      <c r="A60" t="s">
+      <c r="C60" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3">
+      <c r="A61" t="s">
         <v>833</v>
       </c>
-      <c r="B60" t="s">
+      <c r="B61" t="s">
         <v>834</v>
       </c>
-    </row>
-    <row r="61" spans="1:2">
-      <c r="A61" t="s">
+      <c r="C61" t="s">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3">
+      <c r="A62" t="s">
         <v>835</v>
       </c>
-      <c r="B61" t="s">
+      <c r="B62" t="s">
         <v>836</v>
       </c>
-    </row>
-    <row r="62" spans="1:2">
-      <c r="A62" t="s">
+      <c r="C62" t="s">
+        <v>835</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3">
+      <c r="A63" t="s">
         <v>837</v>
       </c>
-      <c r="B62" t="s">
+      <c r="B63" t="s">
         <v>838</v>
       </c>
-    </row>
-    <row r="63" spans="1:2">
-      <c r="A63" t="s">
+      <c r="C63" t="s">
+        <v>926</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3">
+      <c r="A64" t="s">
         <v>839</v>
       </c>
-      <c r="B63" t="s">
+      <c r="B64" t="s">
         <v>840</v>
       </c>
-    </row>
-    <row r="64" spans="1:2">
-      <c r="A64" t="s">
+      <c r="C64" t="s">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3">
+      <c r="A65" t="s">
         <v>841</v>
       </c>
-      <c r="B64" t="s">
+      <c r="B65" t="s">
         <v>842</v>
       </c>
-    </row>
-    <row r="65" spans="1:2">
-      <c r="A65" t="s">
+      <c r="C65" t="s">
+        <v>841</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3">
+      <c r="A66" t="s">
         <v>843</v>
       </c>
-      <c r="B65" t="s">
+      <c r="B66" t="s">
         <v>844</v>
       </c>
-    </row>
-    <row r="66" spans="1:2">
-      <c r="A66" t="s">
+      <c r="C66" t="s">
+        <v>843</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3">
+      <c r="A67" t="s">
         <v>845</v>
       </c>
-      <c r="B66" t="s">
+      <c r="B67" t="s">
         <v>846</v>
       </c>
-    </row>
-    <row r="67" spans="1:2">
-      <c r="A67" t="s">
+      <c r="C67" t="s">
+        <v>845</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3">
+      <c r="A68" t="s">
         <v>847</v>
       </c>
-      <c r="B67" t="s">
+      <c r="B68" t="s">
         <v>848</v>
       </c>
-    </row>
-    <row r="68" spans="1:2">
-      <c r="A68" t="s">
+      <c r="C68" t="s">
+        <v>847</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3">
+      <c r="A69" t="s">
         <v>849</v>
       </c>
-      <c r="B68" t="s">
+      <c r="B69" t="s">
         <v>850</v>
       </c>
-    </row>
-    <row r="69" spans="1:2">
-      <c r="A69" t="s">
+      <c r="C69" t="s">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3">
+      <c r="A70" t="s">
         <v>851</v>
       </c>
-      <c r="B69" t="s">
+      <c r="B70" t="s">
         <v>852</v>
       </c>
-    </row>
-    <row r="70" spans="1:2">
-      <c r="A70" t="s">
+      <c r="C70" t="s">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3">
+      <c r="A71" t="s">
         <v>853</v>
       </c>
-      <c r="B70" t="s">
+      <c r="B71" t="s">
         <v>854</v>
       </c>
-    </row>
-    <row r="71" spans="1:2">
-      <c r="A71" t="s">
+      <c r="C71" t="s">
+        <v>853</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3">
+      <c r="A72" t="s">
         <v>855</v>
       </c>
-      <c r="B71" t="s">
+      <c r="B72" t="s">
+        <v>797</v>
+      </c>
+      <c r="C72" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3">
+      <c r="A73" t="s">
         <v>856</v>
       </c>
-    </row>
-    <row r="72" spans="1:2">
-      <c r="A72" t="s">
+      <c r="B73" t="s">
         <v>857</v>
       </c>
-      <c r="B72" t="s">
-        <v>799</v>
-      </c>
-    </row>
-    <row r="73" spans="1:2">
-      <c r="A73" t="s">
-        <v>858</v>
-      </c>
-      <c r="B73" t="s">
-        <v>859</v>
+      <c r="C73" t="s">
+        <v>856</v>
       </c>
     </row>
   </sheetData>

</xml_diff>